<commit_message>
Update product pages and package downloads
</commit_message>
<xml_diff>
--- a/content/site-copy.xlsx
+++ b/content/site-copy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy" sheetId="1" r:id="R3bb8932fc4054ee5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy" sheetId="1" r:id="R422f750a286d4a14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -850,7 +850,7 @@
         <x:v>products.renamer.downloadUrl</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>https://example.com/download/renamer</x:v>
+        <x:v>../../downloads/slite-clip-renamer-1.0.zip</x:v>
       </x:c>
       <x:c r="D48" t="str">
         <x:v>下载按钮跳转链接</x:v>
@@ -863,90 +863,90 @@
       <x:c r="B49" t="str">
         <x:v>products.renamer.detailPlaceholder</x:v>
       </x:c>
-      <x:c r="C49" t="str">
-        <x:v>这里预留 Renamer 的完整说明书内容。后续你把正式文案发给我后，我会直接把这一整块替换成完整介绍、使用方法和需要补充的技术说明。</x:v>
-      </x:c>
+      <x:c r="C49" t="str"/>
       <x:c r="D49" t="str">
         <x:v>详情页大段说明占位</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>products.exporter.title</x:v>
+        <x:v>products.renamer.detailSections.0.heading</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Exporter</x:v>
+        <x:v>1. 它是什么</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>主标题</x:v>
+        <x:v>可编辑文案</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>products.exporter.subtitle</x:v>
+        <x:v>products.renamer.detailSections.0.body</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>多功能Clips批量导出工具</x:v>
+        <x:v>Renamer 是一个面向 Ableton Live Arrangement View 的批量 clip 重命名工具。它的核心目标不是导出音频，而是在编排阶段先 capture 一组明确的 arrangement clips，再通过规则 preview 结果，最后统一把新名称写回工程。</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>副标题文案</x:v>
+        <x:v>可编辑文案</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>products.exporter.description</x:v>
+        <x:v>products.renamer.detailSections.1.heading</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>多样的导出设置和更方便的Clips多选功能，大幅提升在 Live 内大量导出Clips的效率</x:v>
+        <x:v>2. Capture 如何工作</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>产品简介文案</x:v>
+        <x:v>可编辑文案</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>products.exporter.downloadUrl</x:v>
+        <x:v>products.renamer.detailSections.1.body</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>../../downloads/slite-clip-exporter-1.0.zip</x:v>
+        <x:v>Renamer 通过固定的 capture 方式先建立一组待命名 clips。它只支持两种轨道范围：当前选中轨道，或全部轨道；在此基础上再叠加是否使用当前 loop 范围，于是形成 4 种固定 capture 入口。普通 TRACK / TRACKS 会忽略当前 loop，而两个 IN LOOP 模式只会纳入与当前 loop 区间发生重叠的 clips。</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>下载按钮跳转链接</x:v>
+        <x:v>可编辑文案</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>products.exporter.detailPlaceholder</x:v>
-      </x:c>
-      <x:c r="C54" t="str"/>
+        <x:v>products.renamer.detailSections.2.heading</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>3. 你可以控制什么</x:v>
+      </x:c>
       <x:c r="D54" t="str">
-        <x:v>详情页大段说明占位</x:v>
+        <x:v>可编辑文案</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>products.exporter.detailSections.0.heading</x:v>
+        <x:v>products.renamer.detailSections.2.body</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>1. 它是什么</x:v>
+        <x:v>Renamer 当前可控制的命名规则包括：root、replace、remove、insert、locator、track、index。你可以先 capture，再逐条开启或调整规则，通过 before / after 预览观察变化；真正写回 Live 只会发生在点击 RENAME 之后。</x:v>
       </x:c>
       <x:c r="D55" t="str">
         <x:v>可编辑文案</x:v>
@@ -954,13 +954,13 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>products.exporter.detailSections.0.body</x:v>
+        <x:v>products.renamer.detailSections.3.heading</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>Exporter 是一个面向 Ableton Live Arrangement View 的批量 clip 导出工具。它的工作方式不是任意自由组合轨道，而是先通过 capture 固定本次导出集合，再统一按当前参数批量输出。</x:v>
+        <x:v>4. Preview 的意义</x:v>
       </x:c>
       <x:c r="D56" t="str">
         <x:v>可编辑文案</x:v>
@@ -968,13 +968,13 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>products.exporter.detailSections.1.heading</x:v>
+        <x:v>products.renamer.detailSections.3.body</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>2. Capture 如何工作</x:v>
+        <x:v>before 显示的是 capture 时记录下来的原始名称，after 显示的是当前规则叠加后的目标名称。它们不是两组独立对象，而是同一批已 capture clips 的前后对照。规则、loop、locator 名称或轨道名变化时，preview 会更新；但如果目标集合本身变了，比如新增、删除、移动了 clips，或者你切换到另一组轨道，就必须重新 capture。</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>可编辑文案</x:v>
@@ -982,13 +982,13 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>products.exporter.detailSections.1.body</x:v>
+        <x:v>products.renamer.detailSections.4.heading</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Capture 决定本次要导出的 clips 到底是谁。它只支持两种轨道范围：当前单个选中轨道，或全部轨道；再结合是否叠加 loop 范围，形成 4 种固定 capture 模式：单轨、单轨并叠加 loop、全轨、全轨并叠加 loop。Preview 和 Export 都只会针对这一次 capture 得到的集合生效。</x:v>
+        <x:v>5. 已知边界</x:v>
       </x:c>
       <x:c r="D58" t="str">
         <x:v>可编辑文案</x:v>
@@ -996,13 +996,13 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>products.exporter.detailSections.2.heading</x:v>
+        <x:v>products.renamer.detailSections.4.body</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>3. 你可以控制什么</x:v>
+        <x:v>当前需要注意的边界包括：Renamer 不支持矩阵式任意多轨自由组合命名；IN LOOP 模式要求当前工程已经存在有效 loop；replace 开启但 target 为空时不会产生实际效果；locator 开启但 loop 内没有可归属的 locator 名称时不会按预期生效；此外，如果 capture 后目标范围发生变化，仅改规则并不会自动更新本次命名对象，必须重新 capture。</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>可编辑文案</x:v>
@@ -1010,13 +1010,13 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>products.exporter.detailSections.2.body</x:v>
+        <x:v>products.renamer.detailSections.5.heading</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>当前可控制的导出参数包括：sample rate、bit depth、channel、normalize、peak ceiling、clip gain、export folder，以及用于确认结果的 preview。你可以先 capture，再根据这批 clips 的需要统一调整参数后导出。</x:v>
+        <x:v>6. 状态反馈</x:v>
       </x:c>
       <x:c r="D60" t="str">
         <x:v>可编辑文案</x:v>
@@ -1024,13 +1024,13 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="str">
-        <x:v>product.exporter</x:v>
+        <x:v>product.renamer</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>products.exporter.detailSections.3.heading</x:v>
+        <x:v>products.renamer.detailSections.5.body</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>4. Preview 的意义</x:v>
+        <x:v>Renamer 当前没有像 Exporter 那样独立的彩色状态栏，它的反馈主要通过设备输出消息给出。例如 capture 成功、没有命中目标 clips、loop 不可用、没有 active rules、或 rename 已执行在多少个 clips 上，都会以文字结果提示。可以把这些消息理解为当前动作是否成功、是否需要先检查 loop、轨道范围或规则状态。</x:v>
       </x:c>
       <x:c r="D61" t="str">
         <x:v>可编辑文案</x:v>
@@ -1041,13 +1041,13 @@
         <x:v>product.exporter</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>products.exporter.detailSections.3.body</x:v>
+        <x:v>products.exporter.title</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Preview 显示的不是整个 Arrangement 里的所有 clips，而是本次 capture 之后冻结下来的导出集合。它的作用是帮助你确认当前这次准备导出的内容是否正确；如果你改了轨道、loop、source 或 consolidate 状态，但 preview 没有变化，通常说明你需要重新 capture。</x:v>
+        <x:v>Exporter</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>可编辑文案</x:v>
+        <x:v>主标题</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -1055,13 +1055,13 @@
         <x:v>product.exporter</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>products.exporter.detailSections.4.heading</x:v>
+        <x:v>products.exporter.subtitle</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>5. 已知边界</x:v>
+        <x:v>多功能Clips批量导出工具</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>可编辑文案</x:v>
+        <x:v>副标题文案</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -1069,13 +1069,13 @@
         <x:v>product.exporter</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>products.exporter.detailSections.4.body</x:v>
+        <x:v>products.exporter.description</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>当前需要注意的边界包括：capture 之后如果 source 发生变化，Exporter 会阻止继续导出；fresh consolidate 在不同平台上表现不完全一致，尤其 Windows 更建议保存并重开工程后重新 capture；resample 与 bounce 得到的 clips 在 Windows 上也可能存在差异；如果之前保存的导出路径已经失效，界面会保留旧路径显示，但导出会被阻止，直到你重新选择有效目录。</x:v>
+        <x:v>多样的导出设置和更方便的Clips多选功能，大幅提升在 Live 内大量导出Clips的效率</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>可编辑文案</x:v>
+        <x:v>产品简介文案</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -1083,13 +1083,13 @@
         <x:v>product.exporter</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>products.exporter.detailSections.5.heading</x:v>
+        <x:v>products.exporter.downloadUrl</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>6. 状态反馈</x:v>
+        <x:v>../../downloads/slite-clip-exporter-1.0.zip</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>可编辑文案</x:v>
+        <x:v>下载按钮跳转链接</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -1097,12 +1097,178 @@
         <x:v>product.exporter</x:v>
       </x:c>
       <x:c r="B66" t="str">
+        <x:v>products.exporter.detailPlaceholder</x:v>
+      </x:c>
+      <x:c r="C66" t="str"/>
+      <x:c r="D66" t="str">
+        <x:v>详情页大段说明占位</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>products.exporter.detailSections.0.heading</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>1. 它是什么</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>products.exporter.detailSections.0.body</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>Exporter 是一个面向 Ableton Live Arrangement View 的批量 clip 导出工具。它的工作方式不是任意自由组合轨道，而是先通过 capture 固定本次导出集合，再统一按当前参数批量输出。</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>products.exporter.detailSections.1.heading</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>2. Capture 如何工作</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>products.exporter.detailSections.1.body</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>Exporter 沿用了与 Renamer 一致的 capture 思路：先确定本次要处理的 clips 集合，再统一执行后续操作。它只支持两种轨道范围：当前单个选中轨道，或全部轨道；再结合是否叠加 loop 范围，形成 4 种固定 capture 模式：单轨、单轨并叠加 loop、全轨、全轨并叠加 loop。Preview 和 Export 都只会针对这一次 capture 得到的集合生效。</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>products.exporter.detailSections.2.heading</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>3. 你可以控制什么</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>products.exporter.detailSections.2.body</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>当前可控制的导出参数包括：sample rate、bit depth、channel、normalize、peak ceiling、clip gain、export folder，以及用于确认结果的 preview。你可以先 capture，再根据这批 clips 的需要统一调整参数后导出。</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>products.exporter.detailSections.3.heading</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>4. Preview 的意义</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>products.exporter.detailSections.3.body</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Preview 显示的不是整个 Arrangement 里的所有 clips，而是本次 capture 之后冻结下来的导出集合。它的作用是帮助你确认当前这次准备导出的内容是否正确；如果你改了轨道、loop、source 或 consolidate 状态，但 preview 没有变化，通常说明你需要重新 capture。</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>products.exporter.detailSections.4.heading</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>5. 已知边界</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>products.exporter.detailSections.4.body</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>当前需要注意的边界包括：capture 之后如果 source 发生变化，Exporter 会阻止继续导出；fresh consolidate 在不同平台上表现不完全一致，尤其 Windows 更建议保存并重开工程后重新 capture；resample 与 bounce 得到的 clips 在 Windows 上也可能存在差异；如果之前保存的导出路径已经失效，界面会保留旧路径显示，但导出会被阻止，直到你重新选择有效目录。</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>products.exporter.detailSections.5.heading</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>6. 状态反馈</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>可编辑文案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>product.exporter</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
         <x:v>products.exporter.detailSections.5.body</x:v>
       </x:c>
-      <x:c r="C66" t="str">
+      <x:c r="C78" t="str">
         <x:v>Exporter 用三种颜色提示当前状态：红色表示 error，需要先处理问题；绿色表示 success，说明本次导出已经完成；黄色表示 notice，通常是像重名 clip 这样的提醒，不会阻止导出，但值得你注意。</x:v>
       </x:c>
-      <x:c r="D66" t="str">
+      <x:c r="D78" t="str">
         <x:v>可编辑文案</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add bilingual site and language routing
</commit_message>
<xml_diff>
--- a/content/site-copy.xlsx
+++ b/content/site-copy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy" sheetId="1" r:id="R422f750a286d4a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy" sheetId="1" r:id="R727dec2c6bfc4327"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,7 +354,7 @@
         <x:v>footer.legalLabel</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Legal</x:v>
+        <x:v>Policies</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>可编辑文案</x:v>
@@ -544,7 +544,7 @@
         <x:v>pages.legal.pageTitle</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>Legal / slite.audio</x:v>
+        <x:v>Policies / slite.audio</x:v>
       </x:c>
       <x:c r="D26" t="str">
         <x:v>浏览器标签页标题</x:v>
@@ -584,7 +584,7 @@
         <x:v>pages.legal.title</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>Legal</x:v>
+        <x:v>Policies</x:v>
       </x:c>
       <x:c r="D29" t="str">
         <x:v>主标题</x:v>

</xml_diff>

<commit_message>
Refine homepage M4L headline copy
</commit_message>
<xml_diff>
--- a/content/site-copy.xlsx
+++ b/content/site-copy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy" sheetId="1" r:id="R727dec2c6bfc4327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy" sheetId="1" r:id="Rdd9c9610c1b248a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -283,7 +283,7 @@
         <x:v>site.home.title</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Slite's Max Tools</x:v>
+        <x:v>Slite's M4L Tools</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>主标题</x:v>
@@ -297,8 +297,8 @@
         <x:v>site.home.subtitle</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>两个能让你在Arrangment View里
-畅快地进行批量操作的Max for Live</x:v>
+        <x:v>两款Max for Live让你在Arrangment View里
+畅快地进行批量操作</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>副标题文案</x:v>

</xml_diff>